<commit_message>
fix: remove worksheet protection from home bakery workbook - no password prompts
</commit_message>
<xml_diff>
--- a/digital-products/home-bakery-calculator/singapore-home-bakery-pricing-profit-calculator-2026.xlsx
+++ b/digital-products/home-bakery-calculator/singapore-home-bakery-pricing-profit-calculator-2026.xlsx
@@ -707,7 +707,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -742,51 +742,37 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -809,9 +795,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -819,12 +804,8 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
@@ -835,28 +816,20 @@
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1419,7 +1392,6 @@
       <c r="F29" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="22">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
@@ -1883,7 +1855,6 @@
       <c r="G29" s="22"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="3">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
@@ -1953,151 +1924,151 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="24">
+      <c r="C4" s="23">
         <v>300</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="25">
         <f>$C4*'INGREDIENTS'!F4</f>
         <v>0</v>
       </c>
-      <c r="F4" s="27" t="str">
+      <c r="F4" s="26" t="str">
         <f>IF($E$10=0,"",E4/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="24">
+      <c r="C5" s="23">
         <v>200</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="25">
         <f>$C5*'INGREDIENTS'!F5</f>
         <v>0</v>
       </c>
-      <c r="F5" s="27" t="str">
+      <c r="F5" s="26" t="str">
         <f>IF($E$10=0,"",E5/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="24">
+      <c r="C6" s="23">
         <v>100</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="25">
         <f>$C6*'INGREDIENTS'!F6</f>
         <v>0</v>
       </c>
-      <c r="F6" s="27" t="str">
+      <c r="F6" s="26" t="str">
         <f>IF($E$10=0,"",E6/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="23">
         <v>1</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="25">
         <f>$C7*'INGREDIENTS'!F8</f>
         <v>0</v>
       </c>
-      <c r="F7" s="27" t="str">
+      <c r="F7" s="26" t="str">
         <f>IF($E$10=0,"",E7/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="23">
         <v>5</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="25">
         <f>$C8*'INGREDIENTS'!F9</f>
         <v>0</v>
       </c>
-      <c r="F8" s="27" t="str">
+      <c r="F8" s="26" t="str">
         <f>IF($E$10=0,"",E8/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="23">
         <v>2</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="25">
         <f>$C9*'INGREDIENTS'!F11</f>
         <v>0</v>
       </c>
-      <c r="F9" s="27" t="str">
+      <c r="F9" s="26" t="str">
         <f>IF($E$10=0,"",E9/$E$10)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29">
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="28">
         <f>SUM(E4:E9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="31">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="30" t="s">
         <v>65</v>
       </c>
       <c r="C14" s="15">
@@ -2105,10 +2076,10 @@
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <f>C13*C14</f>
         <v>0</v>
       </c>
@@ -2124,7 +2095,6 @@
       <c r="G17" s="22"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="5">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
@@ -2174,165 +2144,164 @@
       <c r="H2" s="9"/>
     </row>
     <row r="4" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="12" t="s">
         <v>71</v>
       </c>
       <c r="C5" s="15">
         <v>18</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="17" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="34">
         <v>2.5</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="17" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="12" t="s">
         <v>76</v>
       </c>
       <c r="C8" s="15">
         <v>2.8</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="17" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="12" t="s">
         <v>79</v>
       </c>
       <c r="C10" s="15">
         <v>25</v>
       </c>
-      <c r="D10" s="35" t="s">
+      <c r="D10" s="17" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="12" t="s">
         <v>81</v>
       </c>
       <c r="C11" s="15">
         <v>30</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="17" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="31">
         <v>20</v>
       </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="17" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <f>C5*C6</f>
         <v>0</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="17" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="33">
+      <c r="C16" s="32">
         <f>C10+C11</f>
         <v>0</v>
       </c>
-      <c r="D16" s="35" t="s">
+      <c r="D16" s="17" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="32">
         <f>IF(C12=0,0,C16/C12)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="35" t="s">
+      <c r="D17" s="17" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="32">
         <f>C8+C17</f>
         <v>0</v>
       </c>
-      <c r="D18" s="35" t="s">
+      <c r="D18" s="17" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="6">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
@@ -2383,207 +2352,206 @@
       <c r="H2" s="9"/>
     </row>
     <row r="4" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="33">
+      <c r="C5" s="32">
         <f>'RECIPE COSTING'!E10</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="25">
         <f>'RECIPE COSTING'!C15</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="25">
         <f>'LABOUR &amp; OVERHEAD'!C15</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="25">
         <f>'LABOUR &amp; OVERHEAD'!C18</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="36">
         <f>C5+C6+C7+C8</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="39">
+      <c r="C10" s="37">
         <f>'RECIPE COSTING'!C13</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="36">
         <f>IF(C10=0,0,C9/C10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C14" s="40">
+      <c r="C14" s="38">
         <v>0.45</v>
       </c>
-      <c r="D14" s="35" t="s">
+      <c r="D14" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <f>IF(C11=0,0,C11/(1-C14))</f>
         <v>0</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="17" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C16" s="15">
         <v>4.5</v>
       </c>
-      <c r="D16" s="35" t="s">
+      <c r="D16" s="17" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="25">
         <f>C16-C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="41">
+      <c r="C18" s="39">
         <f>IF(C16=0,0,(C16-C11)/C16)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="25">
         <f>(C16-C11)*C10</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="C22" s="42">
+      <c r="C22" s="40">
         <v>240</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="39">
+      <c r="C23" s="37">
         <f>IF(C10=0,0,ROUNDUP(C22/C10,0))</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="38">
+      <c r="C24" s="36">
         <f>(C16-C11)*C22</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="25">
         <f>C16*C22</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="43" t="str">
+      <c r="B27" s="41" t="str">
         <f>IF(C18&lt;0.3,"⚠ Your margin is below 30% — most home bakeries need 40%+ to survive fees, wastage and slow weeks.","Margin looks workable — remember platform/payment fees (~2–4%) come out of this.")</f>
         <v/>
       </c>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="6">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
@@ -2634,85 +2602,85 @@
       <c r="H2" s="9"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="45">
+      <c r="C4" s="15">
         <f>'PRICING &amp; PROFIT'!C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="12" t="s">
         <v>122</v>
       </c>
       <c r="C5" s="15">
         <v>25</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="17" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="34">
         <v>1.5</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="17" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="12" t="s">
         <v>126</v>
       </c>
       <c r="C7" s="15">
         <v>150</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D7" s="17" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="31">
         <v>24</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="38">
         <f>'PRICING &amp; PROFIT'!C14</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
@@ -2729,48 +2697,47 @@
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="C13" s="47">
+      <c r="C13" s="43">
         <f>'PRICING &amp; PROFIT'!C11</f>
         <v>0</v>
       </c>
-      <c r="D13" s="48" t="str">
+      <c r="D13" s="44" t="str">
         <f>IF(AND('PRICING &amp; PROFIT'!C16-C13&gt;0,'LABOUR &amp; OVERHEAD'!C16&gt;0),'LABOUR &amp; OVERHEAD'!C16/('PRICING &amp; PROFIT'!C16-C13),"n/a")</f>
         <v/>
       </c>
-      <c r="E13" s="35" t="s">
+      <c r="E13" s="17" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="30" t="s">
         <v>136</v>
       </c>
-      <c r="C14" s="47">
+      <c r="C14" s="43">
         <f>C13+C5*C6/MAX(1,'RECIPE COSTING'!13)+C7/MAX(1,C8*'RECIPE COSTING'!13)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="48" t="str">
+      <c r="D14" s="44" t="str">
         <f>IF(('PRICING &amp; PROFIT'!C16-C14)&lt;=0,"price too low",(C7+'LABOUR &amp; OVERHEAD'!C16)/('PRICING &amp; PROFIT'!C16-C14))</f>
         <v/>
       </c>
-      <c r="E14" s="35" t="s">
+      <c r="E14" s="17" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="49" t="str">
+      <c r="B16" s="45" t="str">
         <f>IF(C14&gt;='PRICING &amp; PROFIT'!C16,"Upgrade NOT viable at current price — raise price or negotiate kitchen rates.",IF(C14&lt;='PRICING &amp; PROFIT'!C16*(1-C9),"Upgrade CAN hold your target margin at current price.","Upgrade possible but margin shrinks below target — needs higher price or volume."))</f>
         <v/>
       </c>
-      <c r="C16" s="49"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="5">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
@@ -2825,34 +2792,34 @@
       <c r="C3" s="4"/>
     </row>
     <row r="4" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="46" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="50"/>
+      <c r="C4" s="46"/>
     </row>
     <row r="5" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="50"/>
+      <c r="C5" s="46"/>
     </row>
     <row r="6" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="C6" s="50"/>
+      <c r="C6" s="46"/>
     </row>
     <row r="7" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="C7" s="50"/>
+      <c r="C7" s="46"/>
     </row>
     <row r="8" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="46" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="50"/>
+      <c r="C8" s="46"/>
     </row>
     <row r="10" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
@@ -2861,40 +2828,40 @@
       <c r="C10" s="4"/>
     </row>
     <row r="11" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="50" t="s">
+      <c r="B11" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="C11" s="50"/>
+      <c r="C11" s="46"/>
     </row>
     <row r="12" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="50" t="s">
+      <c r="B12" s="46" t="s">
         <v>148</v>
       </c>
-      <c r="C12" s="50"/>
+      <c r="C12" s="46"/>
     </row>
     <row r="13" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="50" t="s">
+      <c r="B13" s="46" t="s">
         <v>149</v>
       </c>
-      <c r="C13" s="50"/>
+      <c r="C13" s="46"/>
     </row>
     <row r="14" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="46" t="s">
         <v>150</v>
       </c>
-      <c r="C14" s="50"/>
+      <c r="C14" s="46"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="50" t="s">
+      <c r="B15" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="C15" s="50"/>
+      <c r="C15" s="46"/>
     </row>
     <row r="16" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="50" t="s">
+      <c r="B16" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="C16" s="50"/>
+      <c r="C16" s="46"/>
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
@@ -2903,28 +2870,28 @@
       <c r="C18" s="4"/>
     </row>
     <row r="19" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="50" t="s">
+      <c r="B19" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="C19" s="50"/>
+      <c r="C19" s="46"/>
     </row>
     <row r="20" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="50" t="s">
+      <c r="B20" s="46" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="50"/>
+      <c r="C20" s="46"/>
     </row>
     <row r="21" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="46" t="s">
         <v>156</v>
       </c>
-      <c r="C21" s="50"/>
+      <c r="C21" s="46"/>
     </row>
     <row r="22" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="50" t="s">
+      <c r="B22" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="C22" s="50"/>
+      <c r="C22" s="46"/>
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
@@ -2933,25 +2900,24 @@
       <c r="C24" s="4"/>
     </row>
     <row r="25" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="C25" s="50"/>
+      <c r="C25" s="46"/>
     </row>
     <row r="26" ht="32" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="46" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="50"/>
+      <c r="C26" s="46"/>
     </row>
     <row r="27" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="C27" s="50"/>
+      <c r="C27" s="46"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
   <mergeCells count="24">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>

</xml_diff>